<commit_message>
Fase 5 ejecutada: P1/P2, P1-E4, P3 y P5 con su clasificación; sensibilidades del ciclo vital; documento y afirmaciones actualizados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja66M5TMoQNzqNwDgvFAsk
</commit_message>
<xml_diff>
--- a/output/f7/tablas_m1.xlsx
+++ b/output/f7/tablas_m1.xlsx
@@ -4155,480 +4155,1005 @@
     </comment>
     <comment ref="B233" authorId="0" shapeId="0">
       <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C233" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D233" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B234" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C234" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D234" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B235" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C235" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D235" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B236" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C236" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D236" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B237" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C237" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D237" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B238" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C238" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D238" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B239" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C239" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D239" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B240" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C240" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D240" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B241" authorId="0" shapeId="0">
+      <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C233" authorId="0" shapeId="0">
+    <comment ref="C241" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D233" authorId="0" shapeId="0">
+    <comment ref="D241" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B234" authorId="0" shapeId="0">
+    <comment ref="B242" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C234" authorId="0" shapeId="0">
+    <comment ref="C242" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D234" authorId="0" shapeId="0">
+    <comment ref="D242" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B235" authorId="0" shapeId="0">
+    <comment ref="B243" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C235" authorId="0" shapeId="0">
+    <comment ref="C243" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D235" authorId="0" shapeId="0">
+    <comment ref="D243" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B236" authorId="0" shapeId="0">
+    <comment ref="B244" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C236" authorId="0" shapeId="0">
+    <comment ref="C244" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D236" authorId="0" shapeId="0">
+    <comment ref="D244" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B237" authorId="0" shapeId="0">
+    <comment ref="B245" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C237" authorId="0" shapeId="0">
+    <comment ref="C245" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D237" authorId="0" shapeId="0">
+    <comment ref="D245" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B238" authorId="0" shapeId="0">
+    <comment ref="B246" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C238" authorId="0" shapeId="0">
+    <comment ref="C246" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D238" authorId="0" shapeId="0">
+    <comment ref="D246" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B239" authorId="0" shapeId="0">
+    <comment ref="B247" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C239" authorId="0" shapeId="0">
+    <comment ref="C247" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D239" authorId="0" shapeId="0">
+    <comment ref="D247" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B240" authorId="0" shapeId="0">
+    <comment ref="B248" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C240" authorId="0" shapeId="0">
+    <comment ref="C248" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D240" authorId="0" shapeId="0">
+    <comment ref="D248" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B241" authorId="0" shapeId="0">
+    <comment ref="B249" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C241" authorId="0" shapeId="0">
+    <comment ref="C249" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D241" authorId="0" shapeId="0">
+    <comment ref="D249" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B242" authorId="0" shapeId="0">
+    <comment ref="B250" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C242" authorId="0" shapeId="0">
+    <comment ref="C250" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D242" authorId="0" shapeId="0">
+    <comment ref="D250" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B243" authorId="0" shapeId="0">
+    <comment ref="B251" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C243" authorId="0" shapeId="0">
+    <comment ref="C251" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D243" authorId="0" shapeId="0">
+    <comment ref="D251" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B244" authorId="0" shapeId="0">
+    <comment ref="B252" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C244" authorId="0" shapeId="0">
+    <comment ref="C252" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D244" authorId="0" shapeId="0">
+    <comment ref="D252" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B245" authorId="0" shapeId="0">
+    <comment ref="B253" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C245" authorId="0" shapeId="0">
+    <comment ref="C253" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D245" authorId="0" shapeId="0">
+    <comment ref="D253" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B246" authorId="0" shapeId="0">
+    <comment ref="B254" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="C246" authorId="0" shapeId="0">
+    <comment ref="C254" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="D246" authorId="0" shapeId="0">
+    <comment ref="D254" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
       </text>
     </comment>
-    <comment ref="B247" authorId="0" shapeId="0">
+    <comment ref="B255" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C255" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D255" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B256" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C256" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D256" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B257" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C257" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D257" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B258" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="C258" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="D258" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Perfiles M1 (src/m1/f4_ciclo_vital.py)</t>
+      </text>
+    </comment>
+    <comment ref="B259" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C259" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D259" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B260" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C260" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D260" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B261" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C261" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D261" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B262" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C262" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D262" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B263" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C263" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D263" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B264" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C264" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D264" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B265" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C265" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D265" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
+      </text>
+    </comment>
+    <comment ref="C269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
+      </text>
+    </comment>
+    <comment ref="D269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
+      </text>
+    </comment>
+    <comment ref="B270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B277" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C277" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D277" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B278" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C278" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D278" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B279" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="C279" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="D279" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
+      </text>
+    </comment>
+    <comment ref="B280" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
+      </text>
+    </comment>
+    <comment ref="C280" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
+      </text>
+    </comment>
+    <comment ref="D280" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
+      </text>
+    </comment>
+    <comment ref="B281" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
+      </text>
+    </comment>
+    <comment ref="C281" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
+      </text>
+    </comment>
+    <comment ref="D281" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
+      </text>
+    </comment>
+    <comment ref="B282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C247" authorId="0" shapeId="0">
+    <comment ref="C282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D247" authorId="0" shapeId="0">
+    <comment ref="D282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B248" authorId="0" shapeId="0">
+    <comment ref="B283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C248" authorId="0" shapeId="0">
+    <comment ref="C283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D248" authorId="0" shapeId="0">
+    <comment ref="D283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B249" authorId="0" shapeId="0">
+    <comment ref="B284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C249" authorId="0" shapeId="0">
+    <comment ref="C284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D249" authorId="0" shapeId="0">
+    <comment ref="D284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B250" authorId="0" shapeId="0">
+    <comment ref="B285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C250" authorId="0" shapeId="0">
+    <comment ref="C285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D250" authorId="0" shapeId="0">
+    <comment ref="D285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B251" authorId="0" shapeId="0">
+    <comment ref="B286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C251" authorId="0" shapeId="0">
+    <comment ref="C286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D251" authorId="0" shapeId="0">
+    <comment ref="D286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B252" authorId="0" shapeId="0">
+    <comment ref="B287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C252" authorId="0" shapeId="0">
+    <comment ref="C287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D252" authorId="0" shapeId="0">
+    <comment ref="D287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B253" authorId="0" shapeId="0">
+    <comment ref="B288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C253" authorId="0" shapeId="0">
+    <comment ref="C288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D253" authorId="0" shapeId="0">
+    <comment ref="D288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B254" authorId="0" shapeId="0">
+    <comment ref="B289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C254" authorId="0" shapeId="0">
+    <comment ref="C289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D254" authorId="0" shapeId="0">
+    <comment ref="D289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B255" authorId="0" shapeId="0">
+    <comment ref="B290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C255" authorId="0" shapeId="0">
+    <comment ref="C290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D255" authorId="0" shapeId="0">
+    <comment ref="D290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B256" authorId="0" shapeId="0">
+    <comment ref="B291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C256" authorId="0" shapeId="0">
+    <comment ref="C291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D256" authorId="0" shapeId="0">
+    <comment ref="D291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B257" authorId="0" shapeId="0">
+    <comment ref="B292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C257" authorId="0" shapeId="0">
+    <comment ref="C292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D257" authorId="0" shapeId="0">
+    <comment ref="D292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B258" authorId="0" shapeId="0">
+    <comment ref="B293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C258" authorId="0" shapeId="0">
+    <comment ref="C293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D258" authorId="0" shapeId="0">
+    <comment ref="D293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B259" authorId="0" shapeId="0">
+    <comment ref="B294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C259" authorId="0" shapeId="0">
+    <comment ref="C294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D259" authorId="0" shapeId="0">
+    <comment ref="D294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B260" authorId="0" shapeId="0">
+    <comment ref="B295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C260" authorId="0" shapeId="0">
+    <comment ref="C295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D260" authorId="0" shapeId="0">
+    <comment ref="D295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B261" authorId="0" shapeId="0">
+    <comment ref="B296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C261" authorId="0" shapeId="0">
+    <comment ref="C296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D261" authorId="0" shapeId="0">
+    <comment ref="D296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B262" authorId="0" shapeId="0">
+    <comment ref="B297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C262" authorId="0" shapeId="0">
+    <comment ref="C297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D262" authorId="0" shapeId="0">
+    <comment ref="D297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B263" authorId="0" shapeId="0">
+    <comment ref="B298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C263" authorId="0" shapeId="0">
+    <comment ref="C298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D263" authorId="0" shapeId="0">
+    <comment ref="D298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B264" authorId="0" shapeId="0">
+    <comment ref="B299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C264" authorId="0" shapeId="0">
+    <comment ref="C299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D264" authorId="0" shapeId="0">
+    <comment ref="D299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
@@ -5738,7 +6263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L264"/>
+  <dimension ref="A1:L299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -16515,18 +17040,14 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>F4_VA_España_EDAD_0</t>
+          <t>F4_VA_EQUILIBRADO_España_0</t>
         </is>
       </c>
       <c r="B223" s="2" t="n">
-        <v>-163</v>
-      </c>
-      <c r="C223" s="2" t="n">
-        <v>-219</v>
-      </c>
-      <c r="D223" s="2" t="n">
-        <v>-140</v>
-      </c>
+        <v>-121</v>
+      </c>
+      <c r="C223" s="2" t="n"/>
+      <c r="D223" s="2" t="n"/>
       <c r="E223" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16559,25 +17080,21 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 0 años (comparador; intervalo: descuento y bienes públicos)</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), España, nacimiento</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>F4_VA_España_EDAD_20</t>
+          <t>F4_VA_EQUILIBRADO_España_30</t>
         </is>
       </c>
       <c r="B224" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C224" s="2" t="n">
-        <v>-23</v>
-      </c>
-      <c r="D224" s="2" t="n">
-        <v>52</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C224" s="2" t="n"/>
+      <c r="D224" s="2" t="n"/>
       <c r="E224" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16610,25 +17127,21 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 20 años (comparador; intervalo: descuento y bienes públicos)</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), España, llegada o edad 30</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>F4_VA_España_EDAD_30</t>
+          <t>F4_VA_EQUILIBRADO_Resto_UE_0</t>
         </is>
       </c>
       <c r="B225" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="C225" s="2" t="n">
-        <v>-25</v>
-      </c>
-      <c r="D225" s="2" t="n">
-        <v>71</v>
-      </c>
+        <v>-68</v>
+      </c>
+      <c r="C225" s="2" t="n"/>
+      <c r="D225" s="2" t="n"/>
       <c r="E225" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16651,7 +17164,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -16661,25 +17174,21 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 30 años (comparador; intervalo: descuento y bienes públicos)</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), Resto UE, nacimiento</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>F4_VA_España_EDAD_40</t>
+          <t>F4_VA_EQUILIBRADO_Resto_UE_30</t>
         </is>
       </c>
       <c r="B226" s="2" t="n">
-        <v>-41</v>
-      </c>
-      <c r="C226" s="2" t="n">
-        <v>-111</v>
-      </c>
-      <c r="D226" s="2" t="n">
-        <v>4</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="C226" s="2" t="n"/>
+      <c r="D226" s="2" t="n"/>
       <c r="E226" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16702,7 +17211,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -16712,18 +17221,18 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 40 años (comparador; intervalo: descuento y bienes públicos)</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), Resto UE, llegada o edad 30</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_20</t>
+          <t>F4_VA_EQUILIBRADO_Resto_del_mundo_0</t>
         </is>
       </c>
       <c r="B227" s="2" t="n">
-        <v>17</v>
+        <v>-82</v>
       </c>
       <c r="C227" s="2" t="n"/>
       <c r="D227" s="2" t="n"/>
@@ -16749,7 +17258,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -16759,18 +17268,18 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 20</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), Resto del mundo, nacimiento</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_30</t>
+          <t>F4_VA_EQUILIBRADO_Resto_del_mundo_30</t>
         </is>
       </c>
       <c r="B228" s="2" t="n">
-        <v>38</v>
+        <v>-3</v>
       </c>
       <c r="C228" s="2" t="n"/>
       <c r="D228" s="2" t="n"/>
@@ -16796,7 +17305,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -16806,21 +17315,25 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 30</t>
+          <t>Valor actual del escenario principal con presupuesto equilibrado (se suma cada año el saldo medio por persona de 2024, 1,017 €), Resto del mundo, llegada o edad 30</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_40</t>
+          <t>F4_VA_España_EDAD_0</t>
         </is>
       </c>
       <c r="B229" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="C229" s="2" t="n"/>
-      <c r="D229" s="2" t="n"/>
+        <v>-163</v>
+      </c>
+      <c r="C229" s="2" t="n">
+        <v>-219</v>
+      </c>
+      <c r="D229" s="2" t="n">
+        <v>-140</v>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16843,7 +17356,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>España</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -16853,21 +17366,25 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 40</t>
+          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 0 años (comparador; intervalo: descuento y bienes públicos)</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_20</t>
+          <t>F4_VA_España_EDAD_20</t>
         </is>
       </c>
       <c r="B230" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="C230" s="2" t="n"/>
-      <c r="D230" s="2" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="C230" s="2" t="n">
+        <v>-23</v>
+      </c>
+      <c r="D230" s="2" t="n">
+        <v>52</v>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16890,7 +17407,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>España</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -16900,21 +17417,25 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 20</t>
+          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 20 años (comparador; intervalo: descuento y bienes públicos)</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_30</t>
+          <t>F4_VA_España_EDAD_30</t>
         </is>
       </c>
       <c r="B231" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C231" s="2" t="n"/>
-      <c r="D231" s="2" t="n"/>
+        <v>38</v>
+      </c>
+      <c r="C231" s="2" t="n">
+        <v>-25</v>
+      </c>
+      <c r="D231" s="2" t="n">
+        <v>71</v>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16937,7 +17458,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>España</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -16947,21 +17468,25 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 30</t>
+          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 30 años (comparador; intervalo: descuento y bienes públicos)</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_40</t>
+          <t>F4_VA_España_EDAD_40</t>
         </is>
       </c>
       <c r="B232" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C232" s="2" t="n"/>
-      <c r="D232" s="2" t="n"/>
+        <v>-41</v>
+      </c>
+      <c r="C232" s="2" t="n">
+        <v>-111</v>
+      </c>
+      <c r="D232" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
           <t>miles de € (VA)</t>
@@ -16984,7 +17509,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>España</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -16994,28 +17519,24 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 40</t>
+          <t>Valor actual de la contribución neta de la vida restante de una persona nacida en España de 40 años (comparador; intervalo: descuento y bienes públicos)</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_UE_LLEGADA_0</t>
+          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_20</t>
         </is>
       </c>
       <c r="B233" s="2" t="n">
-        <v>-79</v>
-      </c>
-      <c r="C233" s="2" t="n">
-        <v>-287</v>
-      </c>
-      <c r="D233" s="2" t="n">
-        <v>-48</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C233" s="2" t="n"/>
+      <c r="D233" s="2" t="n"/>
       <c r="E233" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
@@ -17040,33 +17561,29 @@
       </c>
       <c r="K233" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 0 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 20</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_UE_LLEGADA_20</t>
+          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_30</t>
         </is>
       </c>
       <c r="B234" s="2" t="n">
-        <v>-9</v>
-      </c>
-      <c r="C234" s="2" t="n">
-        <v>-99</v>
-      </c>
-      <c r="D234" s="2" t="n">
-        <v>117</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C234" s="2" t="n"/>
+      <c r="D234" s="2" t="n"/>
       <c r="E234" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -17091,33 +17608,29 @@
       </c>
       <c r="K234" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 20 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_UE_LLEGADA_30</t>
+          <t>F4_VA_HASTA64_Resto_UE_LLEGADA_40</t>
         </is>
       </c>
       <c r="B235" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C235" s="2" t="n">
-        <v>-94</v>
-      </c>
-      <c r="D235" s="2" t="n">
-        <v>118</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C235" s="2" t="n"/>
+      <c r="D235" s="2" t="n"/>
       <c r="E235" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -17142,33 +17655,29 @@
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 30 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 40</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_UE_LLEGADA_40</t>
+          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_20</t>
         </is>
       </c>
       <c r="B236" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C236" s="2" t="n">
-        <v>-98</v>
-      </c>
-      <c r="D236" s="2" t="n">
-        <v>83</v>
-      </c>
+        <v>-13</v>
+      </c>
+      <c r="C236" s="2" t="n"/>
+      <c r="D236" s="2" t="n"/>
       <c r="E236" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -17188,38 +17697,34 @@
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 40 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 20</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_del_mundo_LLEGADA_0</t>
+          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_30</t>
         </is>
       </c>
       <c r="B237" s="2" t="n">
-        <v>-93</v>
-      </c>
-      <c r="C237" s="2" t="n">
-        <v>-377</v>
-      </c>
-      <c r="D237" s="2" t="n">
-        <v>-50</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C237" s="2" t="n"/>
+      <c r="D237" s="2" t="n"/>
       <c r="E237" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -17244,33 +17749,29 @@
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 0 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_del_mundo_LLEGADA_20</t>
+          <t>F4_VA_HASTA64_Resto_del_mundo_LLEGADA_40</t>
         </is>
       </c>
       <c r="B238" s="2" t="n">
-        <v>-34</v>
-      </c>
-      <c r="C238" s="2" t="n">
-        <v>-198</v>
-      </c>
-      <c r="D238" s="2" t="n">
-        <v>97</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C238" s="2" t="n"/>
+      <c r="D238" s="2" t="n"/>
       <c r="E238" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -17295,33 +17796,29 @@
       </c>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 20 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Parte del valor actual hasta los 64 años («población joven hoy»), llegada a los 40</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_del_mundo_LLEGADA_30</t>
+          <t>F4_VA_IMPUT_UE_Resto_UE_30</t>
         </is>
       </c>
       <c r="B239" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="C239" s="2" t="n">
-        <v>-174</v>
-      </c>
-      <c r="D239" s="2" t="n">
-        <v>98</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C239" s="2" t="n"/>
+      <c r="D239" s="2" t="n"/>
       <c r="E239" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -17341,38 +17838,34 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 30 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Principal con los tramos de edad suprimidos (&lt; 50 observaciones) rellenados con el perfil nativo sin escalar, Resto UE, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>F4_VA_Resto_del_mundo_LLEGADA_40</t>
+          <t>F4_VA_IMPUT_UE_Resto_del_mundo_30</t>
         </is>
       </c>
       <c r="B240" s="2" t="n">
-        <v>-16</v>
-      </c>
-      <c r="C240" s="2" t="n">
-        <v>-172</v>
-      </c>
-      <c r="D240" s="2" t="n">
-        <v>58</v>
-      </c>
+        <v>-12</v>
+      </c>
+      <c r="C240" s="2" t="n"/>
+      <c r="D240" s="2" t="n"/>
       <c r="E240" t="inlineStr">
         <is>
-          <t>miles de € (VA en 2024)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -17397,29 +17890,33 @@
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 40 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
+          <t>Principal con los tramos de edad suprimidos (&lt; 50 observaciones) rellenados con el perfil nativo sin escalar, Resto del mundo, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_20</t>
+          <t>F4_VA_Resto_UE_LLEGADA_0</t>
         </is>
       </c>
       <c r="B241" s="2" t="n">
-        <v>-29</v>
-      </c>
-      <c r="C241" s="2" t="n"/>
-      <c r="D241" s="2" t="n"/>
+        <v>-79</v>
+      </c>
+      <c r="C241" s="2" t="n">
+        <v>-287</v>
+      </c>
+      <c r="D241" s="2" t="n">
+        <v>-48</v>
+      </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -17444,29 +17941,33 @@
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 20</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 0 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_30</t>
+          <t>F4_VA_Resto_UE_LLEGADA_20</t>
         </is>
       </c>
       <c r="B242" s="2" t="n">
-        <v>-28</v>
-      </c>
-      <c r="C242" s="2" t="n"/>
-      <c r="D242" s="2" t="n"/>
+        <v>-9</v>
+      </c>
+      <c r="C242" s="2" t="n">
+        <v>-99</v>
+      </c>
+      <c r="D242" s="2" t="n">
+        <v>117</v>
+      </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -17491,29 +17992,33 @@
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 30</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 20 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_40</t>
+          <t>F4_VA_Resto_UE_LLEGADA_30</t>
         </is>
       </c>
       <c r="B243" s="2" t="n">
-        <v>-49</v>
-      </c>
-      <c r="C243" s="2" t="n"/>
-      <c r="D243" s="2" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="C243" s="2" t="n">
+        <v>-94</v>
+      </c>
+      <c r="D243" s="2" t="n">
+        <v>118</v>
+      </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -17538,29 +18043,33 @@
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 40</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 30 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_20</t>
+          <t>F4_VA_Resto_UE_LLEGADA_40</t>
         </is>
       </c>
       <c r="B244" s="2" t="n">
-        <v>-117</v>
-      </c>
-      <c r="C244" s="2" t="n"/>
-      <c r="D244" s="2" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="C244" s="2" t="n">
+        <v>-98</v>
+      </c>
+      <c r="D244" s="2" t="n">
+        <v>83</v>
+      </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -17580,34 +18089,38 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 20</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto UE que llega a los 40 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_30</t>
+          <t>F4_VA_Resto_del_mundo_LLEGADA_0</t>
         </is>
       </c>
       <c r="B245" s="2" t="n">
-        <v>-101</v>
-      </c>
-      <c r="C245" s="2" t="n"/>
-      <c r="D245" s="2" t="n"/>
+        <v>-93</v>
+      </c>
+      <c r="C245" s="2" t="n">
+        <v>-377</v>
+      </c>
+      <c r="D245" s="2" t="n">
+        <v>-50</v>
+      </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -17632,29 +18145,33 @@
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 30</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 0 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_40</t>
+          <t>F4_VA_Resto_del_mundo_LLEGADA_20</t>
         </is>
       </c>
       <c r="B246" s="2" t="n">
-        <v>-116</v>
-      </c>
-      <c r="C246" s="2" t="n"/>
-      <c r="D246" s="2" t="n"/>
+        <v>-34</v>
+      </c>
+      <c r="C246" s="2" t="n">
+        <v>-198</v>
+      </c>
+      <c r="D246" s="2" t="n">
+        <v>97</v>
+      </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>miles de € (VA)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -17679,39 +18196,43 @@
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Perfiles M1</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 40</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 20 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_15_34</t>
+          <t>F4_VA_Resto_del_mundo_LLEGADA_30</t>
         </is>
       </c>
       <c r="B247" s="2" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="C247" s="2" t="n"/>
-      <c r="D247" s="2" t="n"/>
+        <v>-13</v>
+      </c>
+      <c r="C247" s="2" t="n">
+        <v>-174</v>
+      </c>
+      <c r="D247" s="2" t="n">
+        <v>98</v>
+      </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -17721,44 +18242,48 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 30 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_35_54</t>
+          <t>F4_VA_Resto_del_mundo_LLEGADA_40</t>
         </is>
       </c>
       <c r="B248" s="2" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="C248" s="2" t="n"/>
-      <c r="D248" s="2" t="n"/>
+        <v>-16</v>
+      </c>
+      <c r="C248" s="2" t="n">
+        <v>-172</v>
+      </c>
+      <c r="D248" s="2" t="n">
+        <v>58</v>
+      </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA en 2024)</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -17768,44 +18293,44 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1 (ECV, EPF, ENSE, cuentas AAPP) y Eurostat</t>
         </is>
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>Valor actual de la contribución neta de por vida de una persona nacida en Resto del mundo que llega a los 40 años (principal: descuento 3 %, sin convergencia adicional, salida con riesgo decreciente calibrado a 6.3 % anual, pensiones devengadas exportables, bienes públicos a coste medio; intervalo: las 72 combinaciones de supuestos)</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_55_74</t>
+          <t>F4_VA_SIN_MIN15_Resto_UE_30</t>
         </is>
       </c>
       <c r="B249" s="2" t="n">
-        <v>0.96</v>
+        <v>2</v>
       </c>
       <c r="C249" s="2" t="n"/>
       <c r="D249" s="2" t="n"/>
       <c r="E249" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -17815,44 +18340,44 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>Principal sin el mínimo de 15 años cotizados para la pensión contributiva, Resto UE, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_15_34</t>
+          <t>F4_VA_SIN_MIN15_Resto_del_mundo_30</t>
         </is>
       </c>
       <c r="B250" s="2" t="n">
-        <v>0.9</v>
+        <v>-19</v>
       </c>
       <c r="C250" s="2" t="n"/>
       <c r="D250" s="2" t="n"/>
       <c r="E250" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -17862,44 +18387,44 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>Principal sin el mínimo de 15 años cotizados para la pensión contributiva, Resto del mundo, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_35_54</t>
+          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_20</t>
         </is>
       </c>
       <c r="B251" s="2" t="n">
-        <v>0.89</v>
+        <v>-29</v>
       </c>
       <c r="C251" s="2" t="n"/>
       <c r="D251" s="2" t="n"/>
       <c r="E251" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -17909,44 +18434,44 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 20</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_55_74</t>
+          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_30</t>
         </is>
       </c>
       <c r="B252" s="2" t="n">
-        <v>0.85</v>
+        <v>-28</v>
       </c>
       <c r="C252" s="2" t="n"/>
       <c r="D252" s="2" t="n"/>
       <c r="E252" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -17956,44 +18481,44 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_15_34</t>
+          <t>F4_VA_SIN_SALIDA_Resto_UE_LLEGADA_40</t>
         </is>
       </c>
       <c r="B253" s="2" t="n">
-        <v>0.6</v>
+        <v>-49</v>
       </c>
       <c r="C253" s="2" t="n"/>
       <c r="D253" s="2" t="n"/>
       <c r="E253" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -18003,44 +18528,44 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 40</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_35_54</t>
+          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_20</t>
         </is>
       </c>
       <c r="B254" s="2" t="n">
-        <v>0.82</v>
+        <v>-117</v>
       </c>
       <c r="C254" s="2" t="n"/>
       <c r="D254" s="2" t="n"/>
       <c r="E254" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -18050,44 +18575,44 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 20</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_55_74</t>
+          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_30</t>
         </is>
       </c>
       <c r="B255" s="2" t="n">
-        <v>2.58</v>
+        <v>-101</v>
       </c>
       <c r="C255" s="2" t="n"/>
       <c r="D255" s="2" t="n"/>
       <c r="E255" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -18097,44 +18622,44 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_15_34</t>
+          <t>F4_VA_SIN_SALIDA_Resto_del_mundo_LLEGADA_40</t>
         </is>
       </c>
       <c r="B256" s="2" t="n">
-        <v>0.9</v>
+        <v>-116</v>
       </c>
       <c r="C256" s="2" t="n"/>
       <c r="D256" s="2" t="n"/>
       <c r="E256" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -18144,44 +18669,44 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>Como el principal pero sin salidas (toda la vida en España), llegada a los 40</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_35_54</t>
+          <t>F4_VA_SIN_SUELO_Resto_UE_30</t>
         </is>
       </c>
       <c r="B257" s="2" t="n">
-        <v>1.16</v>
+        <v>10</v>
       </c>
       <c r="C257" s="2" t="n"/>
       <c r="D257" s="2" t="n"/>
       <c r="E257" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -18191,44 +18716,44 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto UE</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>Principal sin el suelo de pensión no contributiva, Resto UE, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_55_74</t>
+          <t>F4_VA_SIN_SUELO_Resto_del_mundo_30</t>
         </is>
       </c>
       <c r="B258" s="2" t="n">
-        <v>1</v>
+        <v>-13</v>
       </c>
       <c r="C258" s="2" t="n"/>
       <c r="D258" s="2" t="n"/>
       <c r="E258" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>miles de € (VA)</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -18238,297 +18763,2010 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>Resto del mundo</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Perfiles M1</t>
         </is>
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>Principal sin el suelo de pensión no contributiva, Resto del mundo, llegada a los 30</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>F6_POB_CUOTA_FUERA_ECV</t>
+          <t>F5_P1_E1_beta</t>
         </is>
       </c>
       <c r="B259" s="2" t="n">
-        <v>18.5</v>
+        <v>-0.021</v>
       </c>
       <c r="C259" s="2" t="n"/>
       <c r="D259" s="2" t="n"/>
       <c r="E259" t="inlineStr">
         <is>
-          <t>% de la población</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
         <is>
-          <t>ECV (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>Cuota de los nacidos fuera en la población de la ECV (hogares privados)</t>
+          <t>P1-E1: efecto sobre tasa_actividad (MC2E, especificación principal)</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_España</t>
+          <t>F5_P1_E1_p</t>
         </is>
       </c>
       <c r="B260" s="2" t="n">
-        <v>6252</v>
+        <v>0.995</v>
       </c>
       <c r="C260" s="2" t="n"/>
       <c r="D260" s="2" t="n"/>
       <c r="E260" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en España</t>
+          <t>P1-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_Resto_UE</t>
+          <t>F5_P1_E2_beta</t>
         </is>
       </c>
       <c r="B261" s="2" t="n">
-        <v>2813</v>
+        <v>-0.636</v>
       </c>
       <c r="C261" s="2" t="n"/>
       <c r="D261" s="2" t="n"/>
       <c r="E261" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto UE</t>
+          <t>P1-E2: efecto sobre log_ocupados (MC2E, especificación principal)</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_Resto_del_mundo</t>
+          <t>F5_P1_E2_p</t>
         </is>
       </c>
       <c r="B262" s="2" t="n">
-        <v>1927</v>
+        <v>0.158</v>
       </c>
       <c r="C262" s="2" t="n"/>
       <c r="D262" s="2" t="n"/>
       <c r="E262" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto del mundo</t>
+          <t>P1-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>F6_PREST_NO_CONTRIB_CUOTA</t>
+          <t>F5_P1_E3a_beta</t>
         </is>
       </c>
       <c r="B263" s="2" t="n">
-        <v>2.5</v>
+        <v>-0.6889999999999999</v>
       </c>
       <c r="C263" s="2" t="n"/>
       <c r="D263" s="2" t="n"/>
       <c r="E263" t="inlineStr">
         <is>
-          <t>% de las prestaciones monetarias</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>Rentas mínimas, IMV y ayudas a la vivienda sobre el total de prestaciones monetarias (calibradas a COFOG)</t>
+          <t>P1-E3a: efecto sobre tasa_empleo_educ_baja (MC2E, especificación principal)</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>F6_TRABAJO_CUOTA_FUERA</t>
+          <t>F5_P1_E3a_p</t>
         </is>
       </c>
       <c r="B264" s="2" t="n">
-        <v>15.5</v>
+        <v>0.008</v>
       </c>
       <c r="C264" s="2" t="n"/>
       <c r="D264" s="2" t="n"/>
       <c r="E264" t="inlineStr">
         <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>P1-E3a: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>F5_P1_E3b_beta</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="n">
+        <v>-0.029</v>
+      </c>
+      <c r="C265" s="2" t="n"/>
+      <c r="D265" s="2" t="n"/>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>P1-E3b: efecto sobre tasa_empleo_educ_media (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>F5_P1_E3b_p</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="C266" s="2" t="n"/>
+      <c r="D266" s="2" t="n"/>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>P1-E3b: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>F5_P1_E3c_beta</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="C267" s="2" t="n"/>
+      <c r="D267" s="2" t="n"/>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>P1-E3c: efecto sobre tasa_empleo_educ_alta (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>F5_P1_E3c_p</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="C268" s="2" t="n"/>
+      <c r="D268" s="2" t="n"/>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>P1-E3c: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>F5_P1_E4_beta</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C269" s="2" t="n">
+        <v>-0.5620000000000001</v>
+      </c>
+      <c r="D269" s="2" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Δ log salario por punto de cuota</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>2010-2022</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>españoles (nacionalidad)</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>EES y EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>P1-E4 (Borjas): asociación entre la cuota de nacidos fuera en la celda educación × edad y el salario por hora de los españoles (primeras diferencias; IC orientativo por errores agrupados en 15 celdas; p wild bootstrap = 0.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>F5_P1_F_EFECTIVO</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="C270" s="2" t="n"/>
+      <c r="D270" s="2" t="n"/>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>padrón, ECP (INE)</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>F efectivo de primera etapa agrupado por provincia, especificación principal de P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>F5_P1_F_SHOCK</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="C271" s="2" t="n"/>
+      <c r="D271" s="2" t="n"/>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>padrón, ECP (INE)</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>F de primera etapa al nivel del shock (BHJ), especificación principal de P1 (umbral pre-registrado: 10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>F5_P1_H1_beta</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="n">
+        <v>-0.228</v>
+      </c>
+      <c r="C272" s="2" t="n"/>
+      <c r="D272" s="2" t="n"/>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>P1-H1: efecto sobre tasa_empleo (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>F5_P1_H1_p</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="C273" s="2" t="n"/>
+      <c r="D273" s="2" t="n"/>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>P1-H1: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>F5_P1_H2_beta</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="C274" s="2" t="n"/>
+      <c r="D274" s="2" t="n"/>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>P1-H2: efecto sobre tasa_paro (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>F5_P1_H2_p</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="C275" s="2" t="n"/>
+      <c r="D275" s="2" t="n"/>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>P1-H2: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>F5_P2_E1_beta</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C276" s="2" t="n"/>
+      <c r="D276" s="2" t="n"/>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>P2-E1: efecto sobre cuota_nomanual (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>F5_P2_E1_p</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="C277" s="2" t="n"/>
+      <c r="D277" s="2" t="n"/>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>P2-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>F5_P2_E2_beta</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="n">
+        <v>0.499</v>
+      </c>
+      <c r="C278" s="2" t="n"/>
+      <c r="D278" s="2" t="n"/>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>P2-E2: efecto sobre cuota_alta_cualif (MC2E, especificación principal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>F5_P2_E2_p</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="C279" s="2" t="n"/>
+      <c r="D279" s="2" t="n"/>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>p ajustado</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>2005-2022</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>50 provincias</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>nacidos en España</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>padrón, ECP, EPA (INE)</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>P2-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>F5_P3_EDUC_beta</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="n">
+        <v>-0.169</v>
+      </c>
+      <c r="C280" s="2" t="n">
+        <v>-0.752</v>
+      </c>
+      <c r="D280" s="2" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>alumnos por profesor por punto porcentual</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>2016-2022</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>17 CCAA</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>EDUCAbase, ECP y padrón</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>P3 (educación): asociación entre el aumento de la población nacida fuera de 5-19 años y la ratio de alumnos por profesor en centros públicos (MC2E por comunidad; F efectivo = 39.5; p wild bootstrap de la forma reducida = 0.58; IC orientativo por errores agrupados en 17 comunidades)</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>F5_P5_beta</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="n">
+        <v>-0.325</v>
+      </c>
+      <c r="C281" s="2" t="n"/>
+      <c r="D281" s="2" t="n"/>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>pp por pp</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>2021-2024</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>NUTS2 UE-27</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>nativos</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Eurostat (censo 2021, migr_imm3ctb, EU-LFS)</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>P5: asociación entre la llegada de población nacida fuera y la tasa de empleo de los nativos, NUTS2 de la UE-27, 2021-2024 (MC2E leave-one-country-out; p wild bootstrap por país = 0.38; IC: AKM0 con shocks comunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_CONSULTAS_15_34</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="C282" s="2" t="n"/>
+      <c r="D282" s="2" t="n"/>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_CONSULTAS_35_54</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="C283" s="2" t="n"/>
+      <c r="D283" s="2" t="n"/>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_CONSULTAS_55_74</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="C284" s="2" t="n"/>
+      <c r="D284" s="2" t="n"/>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_FAR_15_34</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C285" s="2" t="n"/>
+      <c r="D285" s="2" t="n"/>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_FAR_35_54</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="C286" s="2" t="n"/>
+      <c r="D286" s="2" t="n"/>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_FAR_55_74</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C287" s="2" t="n"/>
+      <c r="D287" s="2" t="n"/>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_15_34</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C288" s="2" t="n"/>
+      <c r="D288" s="2" t="n"/>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_35_54</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="C289" s="2" t="n"/>
+      <c r="D289" s="2" t="n"/>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_55_74</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="C290" s="2" t="n"/>
+      <c r="D290" s="2" t="n"/>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_15_34</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C291" s="2" t="n"/>
+      <c r="D291" s="2" t="n"/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_35_54</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="C292" s="2" t="n"/>
+      <c r="D292" s="2" t="n"/>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_55_74</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C293" s="2" t="n"/>
+      <c r="D293" s="2" t="n"/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>F6_POB_CUOTA_FUERA_ECV</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C294" s="2" t="n"/>
+      <c r="D294" s="2" t="n"/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>% de la población</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>ECV (INE)</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Cuota de los nacidos fuera en la población de la ECV (hogares privados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_España</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="n">
+        <v>6252</v>
+      </c>
+      <c r="C295" s="2" t="n"/>
+      <c r="D295" s="2" t="n"/>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en España</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_Resto_UE</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="n">
+        <v>2813</v>
+      </c>
+      <c r="C296" s="2" t="n"/>
+      <c r="D296" s="2" t="n"/>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Resto UE</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto UE</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_Resto_del_mundo</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="n">
+        <v>1927</v>
+      </c>
+      <c r="C297" s="2" t="n"/>
+      <c r="D297" s="2" t="n"/>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Resto del mundo</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto del mundo</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>F6_PREST_NO_CONTRIB_CUOTA</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C298" s="2" t="n"/>
+      <c r="D298" s="2" t="n"/>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>% de las prestaciones monetarias</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Rentas mínimas, IMV y ayudas a la vivienda sobre el total de prestaciones monetarias (calibradas a COFOG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>F6_TRABAJO_CUOTA_FUERA</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C299" s="2" t="n"/>
+      <c r="D299" s="2" t="n"/>
+      <c r="E299" t="inlineStr">
+        <is>
           <t>% del total</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr">
+      <c r="F299" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr">
+      <c r="H299" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="I264" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="J264" t="inlineStr">
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
         <is>
           <t>nacidos fuera</t>
         </is>
       </c>
-      <c r="K264" t="inlineStr">
+      <c r="K299" t="inlineStr">
         <is>
           <t>ECV (INE) y Eurostat</t>
         </is>
       </c>
-      <c r="L264" t="inlineStr">
+      <c r="L299" t="inlineStr">
         <is>
           <t>Cuota de los nacidos fuera en IRPF del trabajo y cotizaciones sociales (calibradas a las cuentas de las AAPP)</t>
         </is>

</xml_diff>

<commit_message>
P1-E3a: lectura exploratoria a posteriori (literatura, MCO, empleo frente a población, aritmética por nacionalidad); tarea pendiente de la etiqueta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja66M5TMoQNzqNwDgvFAsk
</commit_message>
<xml_diff>
--- a/output/f7/tablas_m1.xlsx
+++ b/output/f7/tablas_m1.xlsx
@@ -4635,915 +4635,1095 @@
     </comment>
     <comment ref="B265" authorId="0" shapeId="0">
       <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C265" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D265" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D266" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D267" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D268" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D269" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D270" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D271" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D272" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D273" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D274" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D275" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="C276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="D276" authorId="0" shapeId="0">
+      <text>
+        <t>Fuente: EPA (INE) (src/m1/f5_x_e3a_lectura.py)</t>
+      </text>
+    </comment>
+    <comment ref="B277" authorId="0" shapeId="0">
+      <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C265" authorId="0" shapeId="0">
+    <comment ref="C277" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D265" authorId="0" shapeId="0">
+    <comment ref="D277" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B266" authorId="0" shapeId="0">
+    <comment ref="B278" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C266" authorId="0" shapeId="0">
+    <comment ref="C278" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D266" authorId="0" shapeId="0">
+    <comment ref="D278" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B267" authorId="0" shapeId="0">
+    <comment ref="B279" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C267" authorId="0" shapeId="0">
+    <comment ref="C279" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D267" authorId="0" shapeId="0">
+    <comment ref="D279" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B268" authorId="0" shapeId="0">
+    <comment ref="B280" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C268" authorId="0" shapeId="0">
+    <comment ref="C280" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D268" authorId="0" shapeId="0">
+    <comment ref="D280" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B269" authorId="0" shapeId="0">
+    <comment ref="B281" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C269" authorId="0" shapeId="0">
+    <comment ref="C281" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D269" authorId="0" shapeId="0">
+    <comment ref="D281" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B270" authorId="0" shapeId="0">
+    <comment ref="B282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C270" authorId="0" shapeId="0">
+    <comment ref="C282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D270" authorId="0" shapeId="0">
+    <comment ref="D282" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B271" authorId="0" shapeId="0">
+    <comment ref="B283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C271" authorId="0" shapeId="0">
+    <comment ref="C283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D271" authorId="0" shapeId="0">
+    <comment ref="D283" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B272" authorId="0" shapeId="0">
+    <comment ref="B284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C272" authorId="0" shapeId="0">
+    <comment ref="C284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D272" authorId="0" shapeId="0">
+    <comment ref="D284" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B273" authorId="0" shapeId="0">
+    <comment ref="B285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C273" authorId="0" shapeId="0">
+    <comment ref="C285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D273" authorId="0" shapeId="0">
+    <comment ref="D285" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B274" authorId="0" shapeId="0">
+    <comment ref="B286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C274" authorId="0" shapeId="0">
+    <comment ref="C286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D274" authorId="0" shapeId="0">
+    <comment ref="D286" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B275" authorId="0" shapeId="0">
+    <comment ref="B287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C275" authorId="0" shapeId="0">
+    <comment ref="C287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D275" authorId="0" shapeId="0">
+    <comment ref="D287" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B276" authorId="0" shapeId="0">
+    <comment ref="B288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C276" authorId="0" shapeId="0">
+    <comment ref="C288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D276" authorId="0" shapeId="0">
+    <comment ref="D288" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B277" authorId="0" shapeId="0">
+    <comment ref="B289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C277" authorId="0" shapeId="0">
+    <comment ref="C289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D277" authorId="0" shapeId="0">
+    <comment ref="D289" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B278" authorId="0" shapeId="0">
+    <comment ref="B290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C278" authorId="0" shapeId="0">
+    <comment ref="C290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D278" authorId="0" shapeId="0">
+    <comment ref="D290" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B279" authorId="0" shapeId="0">
+    <comment ref="B291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
       </text>
     </comment>
-    <comment ref="C279" authorId="0" shapeId="0">
+    <comment ref="C291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
       </text>
     </comment>
-    <comment ref="D279" authorId="0" shapeId="0">
+    <comment ref="D291" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EES y EPA (INE) (src/m1/f5_p1e4_borjas.py)</t>
       </text>
     </comment>
-    <comment ref="B280" authorId="0" shapeId="0">
+    <comment ref="B292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C280" authorId="0" shapeId="0">
+    <comment ref="C292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D280" authorId="0" shapeId="0">
+    <comment ref="D292" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B281" authorId="0" shapeId="0">
+    <comment ref="B293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C281" authorId="0" shapeId="0">
+    <comment ref="C293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D281" authorId="0" shapeId="0">
+    <comment ref="D293" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B282" authorId="0" shapeId="0">
+    <comment ref="B294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C282" authorId="0" shapeId="0">
+    <comment ref="C294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D282" authorId="0" shapeId="0">
+    <comment ref="D294" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B283" authorId="0" shapeId="0">
+    <comment ref="B295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C283" authorId="0" shapeId="0">
+    <comment ref="C295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D283" authorId="0" shapeId="0">
+    <comment ref="D295" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B284" authorId="0" shapeId="0">
+    <comment ref="B296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C284" authorId="0" shapeId="0">
+    <comment ref="C296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D284" authorId="0" shapeId="0">
+    <comment ref="D296" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B285" authorId="0" shapeId="0">
+    <comment ref="B297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C285" authorId="0" shapeId="0">
+    <comment ref="C297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D285" authorId="0" shapeId="0">
+    <comment ref="D297" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B286" authorId="0" shapeId="0">
+    <comment ref="B298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C286" authorId="0" shapeId="0">
+    <comment ref="C298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D286" authorId="0" shapeId="0">
+    <comment ref="D298" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B287" authorId="0" shapeId="0">
+    <comment ref="B299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C287" authorId="0" shapeId="0">
+    <comment ref="C299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D287" authorId="0" shapeId="0">
+    <comment ref="D299" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B288" authorId="0" shapeId="0">
+    <comment ref="B300" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C288" authorId="0" shapeId="0">
+    <comment ref="C300" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D288" authorId="0" shapeId="0">
+    <comment ref="D300" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B289" authorId="0" shapeId="0">
+    <comment ref="B301" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C289" authorId="0" shapeId="0">
+    <comment ref="C301" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D289" authorId="0" shapeId="0">
+    <comment ref="D301" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B290" authorId="0" shapeId="0">
+    <comment ref="B302" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C290" authorId="0" shapeId="0">
+    <comment ref="C302" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D290" authorId="0" shapeId="0">
+    <comment ref="D302" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B291" authorId="0" shapeId="0">
+    <comment ref="B303" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C291" authorId="0" shapeId="0">
+    <comment ref="C303" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D291" authorId="0" shapeId="0">
+    <comment ref="D303" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B292" authorId="0" shapeId="0">
+    <comment ref="B304" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C292" authorId="0" shapeId="0">
+    <comment ref="C304" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D292" authorId="0" shapeId="0">
+    <comment ref="D304" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B293" authorId="0" shapeId="0">
+    <comment ref="B305" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C293" authorId="0" shapeId="0">
+    <comment ref="C305" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D293" authorId="0" shapeId="0">
+    <comment ref="D305" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B294" authorId="0" shapeId="0">
+    <comment ref="B306" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C294" authorId="0" shapeId="0">
+    <comment ref="C306" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D294" authorId="0" shapeId="0">
+    <comment ref="D306" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B295" authorId="0" shapeId="0">
+    <comment ref="B307" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C295" authorId="0" shapeId="0">
+    <comment ref="C307" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D295" authorId="0" shapeId="0">
+    <comment ref="D307" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B296" authorId="0" shapeId="0">
+    <comment ref="B308" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C296" authorId="0" shapeId="0">
+    <comment ref="C308" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D296" authorId="0" shapeId="0">
+    <comment ref="D308" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B297" authorId="0" shapeId="0">
+    <comment ref="B309" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C297" authorId="0" shapeId="0">
+    <comment ref="C309" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D297" authorId="0" shapeId="0">
+    <comment ref="D309" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B298" authorId="0" shapeId="0">
+    <comment ref="B310" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C298" authorId="0" shapeId="0">
+    <comment ref="C310" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D298" authorId="0" shapeId="0">
+    <comment ref="D310" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B299" authorId="0" shapeId="0">
+    <comment ref="B311" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C299" authorId="0" shapeId="0">
+    <comment ref="C311" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D299" authorId="0" shapeId="0">
+    <comment ref="D311" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B300" authorId="0" shapeId="0">
+    <comment ref="B312" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C300" authorId="0" shapeId="0">
+    <comment ref="C312" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D300" authorId="0" shapeId="0">
+    <comment ref="D312" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B301" authorId="0" shapeId="0">
+    <comment ref="B313" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="C301" authorId="0" shapeId="0">
+    <comment ref="C313" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="D301" authorId="0" shapeId="0">
+    <comment ref="D313" authorId="0" shapeId="0">
       <text>
         <t>Fuente: padrón, ECP, EPA (INE) (src/m1/f5_p1_shiftshare.py)</t>
       </text>
     </comment>
-    <comment ref="B302" authorId="0" shapeId="0">
+    <comment ref="B314" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
       </text>
     </comment>
-    <comment ref="C302" authorId="0" shapeId="0">
+    <comment ref="C314" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
       </text>
     </comment>
-    <comment ref="D302" authorId="0" shapeId="0">
+    <comment ref="D314" authorId="0" shapeId="0">
       <text>
         <t>Fuente: EDUCAbase, ECP y padrón (src/m1/f5_p3_servicios.py)</t>
       </text>
     </comment>
-    <comment ref="B303" authorId="0" shapeId="0">
+    <comment ref="B315" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="C303" authorId="0" shapeId="0">
+    <comment ref="C315" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="D303" authorId="0" shapeId="0">
+    <comment ref="D315" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="B304" authorId="0" shapeId="0">
+    <comment ref="B316" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="C304" authorId="0" shapeId="0">
+    <comment ref="C316" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="D304" authorId="0" shapeId="0">
+    <comment ref="D316" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="B305" authorId="0" shapeId="0">
+    <comment ref="B317" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="C305" authorId="0" shapeId="0">
+    <comment ref="C317" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="D305" authorId="0" shapeId="0">
+    <comment ref="D317" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="B306" authorId="0" shapeId="0">
+    <comment ref="B318" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="C306" authorId="0" shapeId="0">
+    <comment ref="C318" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="D306" authorId="0" shapeId="0">
+    <comment ref="D318" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="B307" authorId="0" shapeId="0">
+    <comment ref="B319" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="C307" authorId="0" shapeId="0">
+    <comment ref="C319" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="D307" authorId="0" shapeId="0">
+    <comment ref="D319" authorId="0" shapeId="0">
       <text>
         <t>Fuente: Eurostat (censo 2021, migr_imm3ctb, EU-LFS) (src/m1/f5_p5_europa.py)</t>
       </text>
     </comment>
-    <comment ref="B308" authorId="0" shapeId="0">
+    <comment ref="B320" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C308" authorId="0" shapeId="0">
+    <comment ref="C320" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D308" authorId="0" shapeId="0">
+    <comment ref="D320" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B309" authorId="0" shapeId="0">
+    <comment ref="B321" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C309" authorId="0" shapeId="0">
+    <comment ref="C321" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D309" authorId="0" shapeId="0">
+    <comment ref="D321" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B310" authorId="0" shapeId="0">
+    <comment ref="B322" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C310" authorId="0" shapeId="0">
+    <comment ref="C322" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D310" authorId="0" shapeId="0">
+    <comment ref="D322" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B311" authorId="0" shapeId="0">
+    <comment ref="B323" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C311" authorId="0" shapeId="0">
+    <comment ref="C323" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D311" authorId="0" shapeId="0">
+    <comment ref="D323" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B312" authorId="0" shapeId="0">
+    <comment ref="B324" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C312" authorId="0" shapeId="0">
+    <comment ref="C324" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D312" authorId="0" shapeId="0">
+    <comment ref="D324" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B313" authorId="0" shapeId="0">
+    <comment ref="B325" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C313" authorId="0" shapeId="0">
+    <comment ref="C325" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D313" authorId="0" shapeId="0">
+    <comment ref="D325" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B314" authorId="0" shapeId="0">
+    <comment ref="B326" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C314" authorId="0" shapeId="0">
+    <comment ref="C326" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D314" authorId="0" shapeId="0">
+    <comment ref="D326" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B315" authorId="0" shapeId="0">
+    <comment ref="B327" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C315" authorId="0" shapeId="0">
+    <comment ref="C327" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D315" authorId="0" shapeId="0">
+    <comment ref="D327" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B316" authorId="0" shapeId="0">
+    <comment ref="B328" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C316" authorId="0" shapeId="0">
+    <comment ref="C328" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D316" authorId="0" shapeId="0">
+    <comment ref="D328" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B317" authorId="0" shapeId="0">
+    <comment ref="B329" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C317" authorId="0" shapeId="0">
+    <comment ref="C329" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D317" authorId="0" shapeId="0">
+    <comment ref="D329" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B318" authorId="0" shapeId="0">
+    <comment ref="B330" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C318" authorId="0" shapeId="0">
+    <comment ref="C330" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D318" authorId="0" shapeId="0">
+    <comment ref="D330" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B319" authorId="0" shapeId="0">
+    <comment ref="B331" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C319" authorId="0" shapeId="0">
+    <comment ref="C331" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D319" authorId="0" shapeId="0">
+    <comment ref="D331" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ENSE 2017 (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B320" authorId="0" shapeId="0">
+    <comment ref="B332" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C320" authorId="0" shapeId="0">
+    <comment ref="C332" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D320" authorId="0" shapeId="0">
+    <comment ref="D332" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B321" authorId="0" shapeId="0">
+    <comment ref="B333" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C321" authorId="0" shapeId="0">
+    <comment ref="C333" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D321" authorId="0" shapeId="0">
+    <comment ref="D333" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B322" authorId="0" shapeId="0">
+    <comment ref="B334" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C322" authorId="0" shapeId="0">
+    <comment ref="C334" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D322" authorId="0" shapeId="0">
+    <comment ref="D334" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B323" authorId="0" shapeId="0">
+    <comment ref="B335" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C323" authorId="0" shapeId="0">
+    <comment ref="C335" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D323" authorId="0" shapeId="0">
+    <comment ref="D335" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B324" authorId="0" shapeId="0">
+    <comment ref="B336" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C324" authorId="0" shapeId="0">
+    <comment ref="C336" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D324" authorId="0" shapeId="0">
+    <comment ref="D336" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat COFOG (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="B325" authorId="0" shapeId="0">
+    <comment ref="B337" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="C325" authorId="0" shapeId="0">
+    <comment ref="C337" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
     </comment>
-    <comment ref="D325" authorId="0" shapeId="0">
+    <comment ref="D337" authorId="0" shapeId="0">
       <text>
         <t>Fuente: ECV (INE) y Eurostat (src/m1/f6_afirmaciones.py)</t>
       </text>
@@ -6653,7 +6833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L325"/>
+  <dimension ref="A1:L337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -19452,17 +19632,17 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>F5_P1_E1_beta</t>
+          <t>F5X_E3a_ELAST</t>
         </is>
       </c>
       <c r="B265" s="2" t="n">
-        <v>-0.021</v>
+        <v>-0.18</v>
       </c>
       <c r="C265" s="2" t="n"/>
       <c r="D265" s="2" t="n"/>
       <c r="E265" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>elasticidad</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -19470,11 +19650,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H265" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -19487,7 +19662,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -19497,24 +19672,24 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>P1-E1: asociación con tasa_actividad (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-E3a expresada como elasticidad de la tasa de empleo respecto a la cuota de nacidos fuera, con medias de los años iniciales (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>F5_P1_E1_p</t>
+          <t>F5X_E3a_MCO</t>
         </is>
       </c>
       <c r="B266" s="2" t="n">
-        <v>0.995</v>
+        <v>-0.2</v>
       </c>
       <c r="C266" s="2" t="n"/>
       <c r="D266" s="2" t="n"/>
       <c r="E266" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -19534,7 +19709,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -19544,24 +19719,24 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>P1-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-E3a por MCO con la especificación principal (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>F5_P1_E2_beta</t>
+          <t>F5X_E3a_OCU</t>
         </is>
       </c>
       <c r="B267" s="2" t="n">
-        <v>-0.636</v>
+        <v>-2.58</v>
       </c>
       <c r="C267" s="2" t="n"/>
       <c r="D267" s="2" t="n"/>
       <c r="E267" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>log por pp</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -19569,11 +19744,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G267" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H267" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -19586,7 +19756,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -19596,18 +19766,18 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>P1-E2: asociación con log_ocupados (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>Δ log ocupados nacidos en España con educación baja por punto de tratamiento, MC2E (exploratorio, a posteriori; p AKM0 sin ajustar = 0.02)</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>F5_P1_E2_p</t>
+          <t>F5X_E3a_OCU_p</t>
         </is>
       </c>
       <c r="B268" s="2" t="n">
-        <v>0.189</v>
+        <v>0.021</v>
       </c>
       <c r="C268" s="2" t="n"/>
       <c r="D268" s="2" t="n"/>
@@ -19633,7 +19803,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -19643,24 +19813,24 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>P1-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>p AKM0 sin ajustar de Δ log ocupados nacidos en España con educación baja (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_CONJ_A</t>
+          <t>F5X_E3a_POB</t>
         </is>
       </c>
       <c r="B269" s="2" t="n">
-        <v>-0.85</v>
+        <v>-1.24</v>
       </c>
       <c r="C269" s="2" t="n"/>
       <c r="D269" s="2" t="n"/>
       <c r="E269" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>log por pp</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -19690,24 +19860,24 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>P1-E3a: el conjunto AKM0 es (−∞, a] ∪ [b, ∞); este es a</t>
+          <t>Δ log población nacida en España de 16-64 con educación baja (EPA) por punto de tratamiento, MC2E (exploratorio, a posteriori; p AKM0 sin ajustar = 0.16)</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_CONJ_B</t>
+          <t>F5X_E3a_POB_MA</t>
         </is>
       </c>
       <c r="B270" s="2" t="n">
-        <v>1.81</v>
+        <v>0.63</v>
       </c>
       <c r="C270" s="2" t="n"/>
       <c r="D270" s="2" t="n"/>
       <c r="E270" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>log por pp</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -19737,28 +19907,24 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>P1-E3a: el conjunto AKM0 es (−∞, a] ∪ [b, ∞); este es b</t>
+          <t>Δ log población nacida en España de 16-64 con educación media o alta (EPA) por punto de tratamiento, MC2E (exploratorio, a posteriori; p AKM0 sin ajustar = 0.16)</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_NACIONALIDAD</t>
+          <t>F5X_E3a_POB_MA_p</t>
         </is>
       </c>
       <c r="B271" s="2" t="n">
-        <v>-0.361</v>
-      </c>
-      <c r="C271" s="2" t="n">
-        <v>-1.014</v>
-      </c>
-      <c r="D271" s="2" t="n">
-        <v>-0.257</v>
-      </c>
+        <v>0.164</v>
+      </c>
+      <c r="C271" s="2" t="n"/>
+      <c r="D271" s="2" t="n"/>
       <c r="E271" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -19766,11 +19932,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H271" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -19793,18 +19954,18 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>P1-E3a: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True, convexo = True)</t>
+          <t>p AKM0 sin ajustar de Δ log población nacida en España de 16-64 con educación media o alta (EPA) (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_PERM_p</t>
+          <t>F5X_E3a_POB_p</t>
         </is>
       </c>
       <c r="B272" s="2" t="n">
-        <v>0.082</v>
+        <v>0.158</v>
       </c>
       <c r="C272" s="2" t="n"/>
       <c r="D272" s="2" t="n"/>
@@ -19840,18 +20001,18 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>P1-E3a: p del placebo de permutación de shocks (500 permutaciones)</t>
+          <t>p AKM0 sin ajustar de Δ log población nacida en España de 16-64 con educación baja (EPA) (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_beta</t>
+          <t>F5X_E3b_NAC</t>
         </is>
       </c>
       <c r="B273" s="2" t="n">
-        <v>-0.6889999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="C273" s="2" t="n"/>
       <c r="D273" s="2" t="n"/>
@@ -19865,11 +20026,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G273" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H273" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -19882,7 +20038,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación media</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -19892,24 +20048,24 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>P1-E3a: asociación con tasa_empleo_educ_baja (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-E3b (educación media), variante por nacionalidad (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>F5_P1_E3a_p</t>
+          <t>F5X_E3c_NAC</t>
         </is>
       </c>
       <c r="B274" s="2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="C274" s="2" t="n"/>
       <c r="D274" s="2" t="n"/>
       <c r="E274" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -19929,7 +20085,7 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación alta</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
@@ -19939,18 +20095,18 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>P1-E3a: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-E3c (educación alta), variante por nacionalidad (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>F5_P1_E3b_beta</t>
+          <t>F5X_NAC_IMPLICITO</t>
         </is>
       </c>
       <c r="B275" s="2" t="n">
-        <v>-0.029</v>
+        <v>-0.16</v>
       </c>
       <c r="C275" s="2" t="n"/>
       <c r="D275" s="2" t="n"/>
@@ -19964,11 +20120,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G275" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H275" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -19991,39 +20142,39 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>P1-E3b: asociación con tasa_empleo_educ_media (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>Media ponderada por educación de las estimaciones por nacionalidad de P1-E3a, E3b y E3c (exploratorio, a posteriori)</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>F5_P1_E3b_p</t>
+          <t>F5X_PESO_BAJA</t>
         </is>
       </c>
       <c r="B276" s="2" t="n">
-        <v>0.995</v>
+        <v>48.7</v>
       </c>
       <c r="C276" s="2" t="n"/>
       <c r="D276" s="2" t="n"/>
       <c r="E276" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>% de los nativos de 16-64</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>2005-2022</t>
+          <t>2005, 2009, 2015</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>50 provincias</t>
+          <t>España</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -20033,23 +20184,23 @@
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>EPA (INE)</t>
         </is>
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>P1-E3b: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>Peso de la educación baja entre los nacidos en España de 16-64 (EPA, años iniciales de los periodos)</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>F5_P1_E3c_beta</t>
+          <t>F5_P1_E1_beta</t>
         </is>
       </c>
       <c r="B277" s="2" t="n">
-        <v>0.18</v>
+        <v>-0.021</v>
       </c>
       <c r="C277" s="2" t="n"/>
       <c r="D277" s="2" t="n"/>
@@ -20090,14 +20241,14 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>P1-E3c: asociación con tasa_empleo_educ_alta (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-E1: asociación con tasa_actividad (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>F5_P1_E3c_p</t>
+          <t>F5_P1_E1_p</t>
         </is>
       </c>
       <c r="B278" s="2" t="n">
@@ -20137,28 +20288,24 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>P1-E3c: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>F5_P1_E4_beta</t>
+          <t>F5_P1_E2_beta</t>
         </is>
       </c>
       <c r="B279" s="2" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="C279" s="2" t="n">
-        <v>-0.5620000000000001</v>
-      </c>
-      <c r="D279" s="2" t="n">
-        <v>0.361</v>
-      </c>
+        <v>-0.636</v>
+      </c>
+      <c r="C279" s="2" t="n"/>
+      <c r="D279" s="2" t="n"/>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Δ log salario por punto de cuota</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -20173,44 +20320,44 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>2010-2022</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>españoles (nacionalidad)</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>EES y EPA (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>P1-E4 (Borjas): asociación entre la cuota de nacidos fuera en la celda educación × edad y el salario por hora de los españoles (primeras diferencias; IC orientativo por errores agrupados en 15 celdas; p wild bootstrap = 0.61)</t>
+          <t>P1-E2: asociación con log_ocupados (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>F5_P1_E6_beta</t>
+          <t>F5_P1_E2_p</t>
         </is>
       </c>
       <c r="B280" s="2" t="n">
-        <v>0.426</v>
+        <v>0.189</v>
       </c>
       <c r="C280" s="2" t="n"/>
       <c r="D280" s="2" t="n"/>
       <c r="E280" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -20218,11 +20365,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G280" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H280" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20245,24 +20387,24 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>P1-E6: asociación con log_pob_nativos (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>F5_P1_E6_p</t>
+          <t>F5_P1_E3a_CONJ_A</t>
         </is>
       </c>
       <c r="B281" s="2" t="n">
-        <v>0.995</v>
+        <v>-0.85</v>
       </c>
       <c r="C281" s="2" t="n"/>
       <c r="D281" s="2" t="n"/>
       <c r="E281" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -20282,7 +20424,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -20292,24 +20434,24 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>P1-E6: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-E3a: el conjunto AKM0 es (−∞, a] ∪ [b, ∞); este es a</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>F5_P1_F_EFECTIVO</t>
+          <t>F5_P1_E3a_CONJ_B</t>
         </is>
       </c>
       <c r="B282" s="2" t="n">
-        <v>24.4</v>
+        <v>1.81</v>
       </c>
       <c r="C282" s="2" t="n"/>
       <c r="D282" s="2" t="n"/>
       <c r="E282" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -20329,34 +20471,38 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>padrón, ECP (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>F efectivo de primera etapa agrupado por provincia, especificación principal de P1</t>
+          <t>P1-E3a: el conjunto AKM0 es (−∞, a] ∪ [b, ∞); este es b</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>F5_P1_F_NACIONALIDAD</t>
+          <t>F5_P1_E3a_NACIONALIDAD</t>
         </is>
       </c>
       <c r="B283" s="2" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="C283" s="2" t="n"/>
-      <c r="D283" s="2" t="n"/>
+        <v>-0.361</v>
+      </c>
+      <c r="C283" s="2" t="n">
+        <v>-1.014</v>
+      </c>
+      <c r="D283" s="2" t="n">
+        <v>-0.257</v>
+      </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -20364,6 +20510,11 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H283" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20376,34 +20527,34 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>padrón (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>F de primera etapa al nivel del shock en la variante por nacionalidad</t>
+          <t>P1-E3a: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True, convexo = True)</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>F5_P1_F_SHOCK</t>
+          <t>F5_P1_E3a_PERM_p</t>
         </is>
       </c>
       <c r="B284" s="2" t="n">
-        <v>6.6</v>
+        <v>0.082</v>
       </c>
       <c r="C284" s="2" t="n"/>
       <c r="D284" s="2" t="n"/>
       <c r="E284" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -20423,34 +20574,34 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España con educación baja</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>padrón, ECP (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>F de primera etapa al nivel del shock (BHJ), especificación principal de P1 (umbral pre-registrado: 10)</t>
+          <t>P1-E3a: p del placebo de permutación de shocks (500 permutaciones)</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>F5_P1_F_SIN_TOP3</t>
+          <t>F5_P1_E3a_beta</t>
         </is>
       </c>
       <c r="B285" s="2" t="n">
-        <v>0.21</v>
+        <v>-0.6889999999999999</v>
       </c>
       <c r="C285" s="2" t="n"/>
       <c r="D285" s="2" t="n"/>
       <c r="E285" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -20458,6 +20609,11 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H285" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20470,38 +20626,34 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>padrón (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>F de primera etapa al nivel del shock al excluir los tres orígenes de mayor peso de Rotemberg (prueba no informativa si es &lt; 10)</t>
+          <t>P1-E3a: asociación con tasa_empleo_educ_baja (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>F5_P1_H1_MULT_MED</t>
+          <t>F5_P1_E3a_p</t>
         </is>
       </c>
       <c r="B286" s="2" t="n">
-        <v>-0.416</v>
-      </c>
-      <c r="C286" s="2" t="n">
-        <v>-0.652</v>
-      </c>
-      <c r="D286" s="2" t="n">
-        <v>-0.174</v>
-      </c>
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="C286" s="2" t="n"/>
+      <c r="D286" s="2" t="n"/>
       <c r="E286" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -20509,11 +20661,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H286" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20521,7 +20668,7 @@
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
@@ -20536,24 +20683,24 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>P1-H1: mediana de β en el multiverso pre-registrado (32 especificaciones; intervalo: mínimo y máximo)</t>
+          <t>P1-E3a: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>F5_P1_H1_MULT_NEG</t>
+          <t>F5_P1_E3b_beta</t>
         </is>
       </c>
       <c r="B287" s="2" t="n">
-        <v>32</v>
+        <v>-0.029</v>
       </c>
       <c r="C287" s="2" t="n"/>
       <c r="D287" s="2" t="n"/>
       <c r="E287" t="inlineStr">
         <is>
-          <t>especificaciones</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -20561,6 +20708,11 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H287" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20568,7 +20720,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
@@ -20583,24 +20735,24 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>P1-H1: especificaciones del multiverso con β negativo (de 32)</t>
+          <t>P1-E3b: asociación con tasa_empleo_educ_media (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>F5_P1_H1_MULT_RECHAZA</t>
+          <t>F5_P1_E3b_p</t>
         </is>
       </c>
       <c r="B288" s="2" t="n">
-        <v>0</v>
+        <v>0.995</v>
       </c>
       <c r="C288" s="2" t="n"/>
       <c r="D288" s="2" t="n"/>
       <c r="E288" t="inlineStr">
         <is>
-          <t>especificaciones</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -20615,7 +20767,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
@@ -20630,25 +20782,21 @@
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>P1-H1: especificaciones del multiverso cuyo AKM0 rechaza β = 0 al 5 % sin ajuste (de 32)</t>
+          <t>P1-E3b: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>F5_P1_H1_NACIONALIDAD</t>
+          <t>F5_P1_E3c_beta</t>
         </is>
       </c>
       <c r="B289" s="2" t="n">
-        <v>-0.118</v>
-      </c>
-      <c r="C289" s="2" t="n">
-        <v>-0.622</v>
-      </c>
-      <c r="D289" s="2" t="n">
-        <v>0.677</v>
-      </c>
+        <v>0.18</v>
+      </c>
+      <c r="C289" s="2" t="n"/>
+      <c r="D289" s="2" t="n"/>
       <c r="E289" t="inlineStr">
         <is>
           <t>pp por pp</t>
@@ -20686,24 +20834,24 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>P1-H1: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True)</t>
+          <t>P1-E3c: asociación con tasa_empleo_educ_alta (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>F5_P1_H1_beta</t>
+          <t>F5_P1_E3c_p</t>
         </is>
       </c>
       <c r="B290" s="2" t="n">
-        <v>-0.228</v>
+        <v>0.995</v>
       </c>
       <c r="C290" s="2" t="n"/>
       <c r="D290" s="2" t="n"/>
       <c r="E290" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -20711,11 +20859,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H290" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20738,24 +20881,28 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>P1-H1: asociación con tasa_empleo (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-E3c: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>F5_P1_H1_p</t>
+          <t>F5_P1_E4_beta</t>
         </is>
       </c>
       <c r="B291" s="2" t="n">
-        <v>0.388</v>
-      </c>
-      <c r="C291" s="2" t="n"/>
-      <c r="D291" s="2" t="n"/>
+        <v>-0.1</v>
+      </c>
+      <c r="C291" s="2" t="n">
+        <v>-0.5620000000000001</v>
+      </c>
+      <c r="D291" s="2" t="n">
+        <v>0.361</v>
+      </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>Δ log salario por punto de cuota</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -20763,47 +20910,48 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>2005-2022</t>
+          <t>2010-2022</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>50 provincias</t>
+          <t>España</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>españoles (nacionalidad)</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>EES y EPA (INE)</t>
         </is>
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>P1-H1: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-E4 (Borjas): asociación entre la cuota de nacidos fuera en la celda educación × edad y el salario por hora de los españoles (primeras diferencias; IC orientativo por errores agrupados en 15 celdas; p wild bootstrap = 0.61)</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>F5_P1_H2_MULT_MED</t>
+          <t>F5_P1_E6_beta</t>
         </is>
       </c>
       <c r="B292" s="2" t="n">
-        <v>0.314</v>
-      </c>
-      <c r="C292" s="2" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="D292" s="2" t="n">
-        <v>0.6</v>
-      </c>
+        <v>0.426</v>
+      </c>
+      <c r="C292" s="2" t="n"/>
+      <c r="D292" s="2" t="n"/>
       <c r="E292" t="inlineStr">
         <is>
           <t>pp por pp</t>
@@ -20826,7 +20974,7 @@
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
@@ -20841,24 +20989,24 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>P1-H2: mediana de β en el multiverso pre-registrado (32 especificaciones; intervalo: mínimo y máximo)</t>
+          <t>P1-E6: asociación con log_pob_nativos (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>F5_P1_H2_MULT_NEG</t>
+          <t>F5_P1_E6_p</t>
         </is>
       </c>
       <c r="B293" s="2" t="n">
-        <v>0</v>
+        <v>0.995</v>
       </c>
       <c r="C293" s="2" t="n"/>
       <c r="D293" s="2" t="n"/>
       <c r="E293" t="inlineStr">
         <is>
-          <t>especificaciones</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -20873,7 +21021,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -20888,24 +21036,24 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>P1-H2: especificaciones del multiverso con β negativo (de 32)</t>
+          <t>P1-E6: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>F5_P1_H2_MULT_RECHAZA</t>
+          <t>F5_P1_F_EFECTIVO</t>
         </is>
       </c>
       <c r="B294" s="2" t="n">
-        <v>3</v>
+        <v>24.4</v>
       </c>
       <c r="C294" s="2" t="n"/>
       <c r="D294" s="2" t="n"/>
       <c r="E294" t="inlineStr">
         <is>
-          <t>especificaciones</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -20920,43 +21068,39 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>provincias</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>todos</t>
         </is>
       </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>padrón, ECP (INE)</t>
         </is>
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>P1-H2: especificaciones del multiverso cuyo AKM0 rechaza β = 0 al 5 % sin ajuste (de 32)</t>
+          <t>F efectivo de primera etapa agrupado por provincia, especificación principal de P1</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>F5_P1_H2_NACIONALIDAD</t>
+          <t>F5_P1_F_NACIONALIDAD</t>
         </is>
       </c>
       <c r="B295" s="2" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="C295" s="2" t="n">
-        <v>-0.733</v>
-      </c>
-      <c r="D295" s="2" t="n">
-        <v>1.227</v>
-      </c>
+        <v>11.1</v>
+      </c>
+      <c r="C295" s="2" t="n"/>
+      <c r="D295" s="2" t="n"/>
       <c r="E295" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -20964,11 +21108,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H295" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -20981,34 +21120,34 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>todos</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>padrón (INE)</t>
         </is>
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>P1-H2: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True)</t>
+          <t>F de primera etapa al nivel del shock en la variante por nacionalidad</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>F5_P1_H2_beta</t>
+          <t>F5_P1_F_SHOCK</t>
         </is>
       </c>
       <c r="B296" s="2" t="n">
-        <v>0.282</v>
+        <v>6.6</v>
       </c>
       <c r="C296" s="2" t="n"/>
       <c r="D296" s="2" t="n"/>
       <c r="E296" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -21016,11 +21155,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G296" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H296" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -21033,34 +21167,34 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>todos</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>padrón, ECP (INE)</t>
         </is>
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>P1-H2: asociación con tasa_paro (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>F de primera etapa al nivel del shock (BHJ), especificación principal de P1 (umbral pre-registrado: 10)</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>F5_P1_H2_p</t>
+          <t>F5_P1_F_SIN_TOP3</t>
         </is>
       </c>
       <c r="B297" s="2" t="n">
-        <v>0.388</v>
+        <v>0.21</v>
       </c>
       <c r="C297" s="2" t="n"/>
       <c r="D297" s="2" t="n"/>
       <c r="E297" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -21080,31 +21214,35 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>nacidos en España</t>
+          <t>todos</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
         <is>
-          <t>padrón, ECP, EPA (INE)</t>
+          <t>padrón (INE)</t>
         </is>
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>P1-H2: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>F de primera etapa al nivel del shock al excluir los tres orígenes de mayor peso de Rotemberg (prueba no informativa si es &lt; 10)</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>F5_P2_E1_beta</t>
+          <t>F5_P1_H1_MULT_MED</t>
         </is>
       </c>
       <c r="B298" s="2" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C298" s="2" t="n"/>
-      <c r="D298" s="2" t="n"/>
+        <v>-0.416</v>
+      </c>
+      <c r="C298" s="2" t="n">
+        <v>-0.652</v>
+      </c>
+      <c r="D298" s="2" t="n">
+        <v>-0.174</v>
+      </c>
       <c r="E298" t="inlineStr">
         <is>
           <t>pp por pp</t>
@@ -21127,7 +21265,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>50 provincias</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
@@ -21142,24 +21280,24 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>P2-E1: asociación con cuota_nomanual (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-H1: mediana de β en el multiverso pre-registrado (32 especificaciones; intervalo: mínimo y máximo)</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>F5_P2_E1_p</t>
+          <t>F5_P1_H1_MULT_NEG</t>
         </is>
       </c>
       <c r="B299" s="2" t="n">
-        <v>0.985</v>
+        <v>32</v>
       </c>
       <c r="C299" s="2" t="n"/>
       <c r="D299" s="2" t="n"/>
       <c r="E299" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>especificaciones</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -21174,7 +21312,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>50 provincias</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
@@ -21189,24 +21327,24 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>P2-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-H1: especificaciones del multiverso con β negativo (de 32)</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>F5_P2_E2_beta</t>
+          <t>F5_P1_H1_MULT_RECHAZA</t>
         </is>
       </c>
       <c r="B300" s="2" t="n">
-        <v>0.499</v>
+        <v>0</v>
       </c>
       <c r="C300" s="2" t="n"/>
       <c r="D300" s="2" t="n"/>
       <c r="E300" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>especificaciones</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -21214,11 +21352,6 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G300" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H300" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -21226,7 +21359,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>50 provincias</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -21241,24 +21374,28 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>P2-E2: asociación con cuota_alta_cualif (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
+          <t>P1-H1: especificaciones del multiverso cuyo AKM0 rechaza β = 0 al 5 % sin ajuste (de 32)</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>F5_P2_E2_p</t>
+          <t>F5_P1_H1_NACIONALIDAD</t>
         </is>
       </c>
       <c r="B301" s="2" t="n">
-        <v>0.306</v>
-      </c>
-      <c r="C301" s="2" t="n"/>
-      <c r="D301" s="2" t="n"/>
+        <v>-0.118</v>
+      </c>
+      <c r="C301" s="2" t="n">
+        <v>-0.622</v>
+      </c>
+      <c r="D301" s="2" t="n">
+        <v>0.677</v>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>p ajustado</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -21266,6 +21403,11 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H301" t="inlineStr">
         <is>
           <t>2005-2022</t>
@@ -21288,28 +21430,24 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>P2-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
+          <t>P1-H1: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True)</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>F5_P3_EDUC_beta</t>
+          <t>F5_P1_H1_beta</t>
         </is>
       </c>
       <c r="B302" s="2" t="n">
-        <v>-0.169</v>
-      </c>
-      <c r="C302" s="2" t="n">
-        <v>-0.752</v>
-      </c>
-      <c r="D302" s="2" t="n">
-        <v>0.414</v>
-      </c>
+        <v>-0.228</v>
+      </c>
+      <c r="C302" s="2" t="n"/>
+      <c r="D302" s="2" t="n"/>
       <c r="E302" t="inlineStr">
         <is>
-          <t>alumnos por profesor por punto porcentual</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -21324,44 +21462,44 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>2016-2022</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>17 CCAA</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>EDUCAbase, ECP y padrón</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>P3 (educación): asociación entre el aumento de la población nacida fuera de 5-19 años y la ratio de alumnos por profesor en centros públicos (MC2E por comunidad; F efectivo = 39.5; p wild bootstrap de la forma reducida = 0.58; IC orientativo por errores agrupados en 17 comunidades)</t>
+          <t>P1-H1: asociación con tasa_empleo (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>F5_P5_HET_centro_y_este</t>
+          <t>F5_P1_H1_p</t>
         </is>
       </c>
       <c r="B303" s="2" t="n">
-        <v>0.027</v>
+        <v>0.388</v>
       </c>
       <c r="C303" s="2" t="n"/>
       <c r="D303" s="2" t="n"/>
       <c r="E303" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -21369,48 +21507,47 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G303" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>NUTS2, centro y este</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>nativos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t>P5, países centro y este: β leave-one-country-out (28 regiones; p wild bootstrap = 0.94)</t>
+          <t>P1-H1: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>F5_P5_HET_continentales</t>
+          <t>F5_P1_H2_MULT_MED</t>
         </is>
       </c>
       <c r="B304" s="2" t="n">
-        <v>-0.163</v>
-      </c>
-      <c r="C304" s="2" t="n"/>
-      <c r="D304" s="2" t="n"/>
+        <v>0.314</v>
+      </c>
+      <c r="C304" s="2" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="D304" s="2" t="n">
+        <v>0.6</v>
+      </c>
       <c r="E304" t="inlineStr">
         <is>
           <t>pp por pp</t>
@@ -21428,44 +21565,44 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>NUTS2, continentales</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>nativos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>P5, países continentales: β leave-one-country-out (93 regiones; p wild bootstrap = 0.80)</t>
+          <t>P1-H2: mediana de β en el multiverso pre-registrado (32 especificaciones; intervalo: mínimo y máximo)</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>F5_P5_HET_mediterráneos</t>
+          <t>F5_P1_H2_MULT_NEG</t>
         </is>
       </c>
       <c r="B305" s="2" t="n">
-        <v>-0.501</v>
+        <v>0</v>
       </c>
       <c r="C305" s="2" t="n"/>
       <c r="D305" s="2" t="n"/>
       <c r="E305" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>especificaciones</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -21473,51 +21610,46 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G305" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>NUTS2, mediterráneos</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>nativos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>P5, países mediterráneos: β leave-one-country-out (57 regiones; p wild bootstrap = 0.31)</t>
+          <t>P1-H2: especificaciones del multiverso con β negativo (de 32)</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>F5_P5_HET_nórdicos</t>
+          <t>F5_P1_H2_MULT_RECHAZA</t>
         </is>
       </c>
       <c r="B306" s="2" t="n">
-        <v>-0.904</v>
+        <v>3</v>
       </c>
       <c r="C306" s="2" t="n"/>
       <c r="D306" s="2" t="n"/>
       <c r="E306" t="inlineStr">
         <is>
-          <t>pp por pp</t>
+          <t>especificaciones</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -21525,51 +21657,46 @@
           <t>C4</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN</t>
-        </is>
-      </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>NUTS2, nórdicos</t>
+          <t>provincias</t>
         </is>
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>nativos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>P5, países nórdicos: β leave-one-country-out (17 regiones; p wild bootstrap = 0.33)</t>
+          <t>P1-H2: especificaciones del multiverso cuyo AKM0 rechaza β = 0 al 5 % sin ajuste (de 32)</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>F5_P5_beta</t>
+          <t>F5_P1_H2_NACIONALIDAD</t>
         </is>
       </c>
       <c r="B307" s="2" t="n">
-        <v>-0.325</v>
+        <v>0.181</v>
       </c>
       <c r="C307" s="2" t="n">
-        <v>-0.968</v>
+        <v>-0.733</v>
       </c>
       <c r="D307" s="2" t="n">
-        <v>0.318</v>
+        <v>1.227</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -21588,44 +21715,44 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>NUTS2 UE-27</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>nativos</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>Eurostat (censo 2021, migr_imm3ctb, EU-LFS)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>P5: asociación entre la llegada de población nacida fuera y la tasa de empleo de los nativos, NUTS2 de la UE-27, 2021-2024 (MC2E leave-one-country-out; p wild bootstrap por país = 0.38; IC orientativo por errores agrupados por país)</t>
+          <t>P1-H2: variante con instrumento y tratamiento por nacionalidad (F al nivel del shock = 11.1; IC: conjunto AKM0, acotado = True)</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_15_34</t>
+          <t>F5_P1_H2_beta</t>
         </is>
       </c>
       <c r="B308" s="2" t="n">
-        <v>1.02</v>
+        <v>0.282</v>
       </c>
       <c r="C308" s="2" t="n"/>
       <c r="D308" s="2" t="n"/>
       <c r="E308" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -21633,46 +21760,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>P1-H2: asociación con tasa_paro (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_35_54</t>
+          <t>F5_P1_H2_p</t>
         </is>
       </c>
       <c r="B309" s="2" t="n">
-        <v>0.84</v>
+        <v>0.388</v>
       </c>
       <c r="C309" s="2" t="n"/>
       <c r="D309" s="2" t="n"/>
       <c r="E309" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -21682,44 +21814,44 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>P1-H2: p de AKM0 frente a β = 0 ajustado (Holm); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_CONSULTAS_55_74</t>
+          <t>F5_P2_E1_beta</t>
         </is>
       </c>
       <c r="B310" s="2" t="n">
-        <v>0.96</v>
+        <v>0.025</v>
       </c>
       <c r="C310" s="2" t="n"/>
       <c r="D310" s="2" t="n"/>
       <c r="E310" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -21727,46 +21859,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>P2-E1: asociación con cuota_nomanual (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_15_34</t>
+          <t>F5_P2_E1_p</t>
         </is>
       </c>
       <c r="B311" s="2" t="n">
-        <v>0.9</v>
+        <v>0.985</v>
       </c>
       <c r="C311" s="2" t="n"/>
       <c r="D311" s="2" t="n"/>
       <c r="E311" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -21776,44 +21913,44 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J311" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>P2-E1: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_35_54</t>
+          <t>F5_P2_E2_beta</t>
         </is>
       </c>
       <c r="B312" s="2" t="n">
-        <v>0.89</v>
+        <v>0.499</v>
       </c>
       <c r="C312" s="2" t="n"/>
       <c r="D312" s="2" t="n"/>
       <c r="E312" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -21821,46 +21958,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>P2-E2: asociación con cuota_alta_cualif (MC2E, especificación principal; IC: envolvente del conjunto AKM0)</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_FAR_55_74</t>
+          <t>F5_P2_E2_p</t>
         </is>
       </c>
       <c r="B313" s="2" t="n">
-        <v>0.85</v>
+        <v>0.306</v>
       </c>
       <c r="C313" s="2" t="n"/>
       <c r="D313" s="2" t="n"/>
       <c r="E313" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>p ajustado</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -21870,44 +22012,48 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2005-2022</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>50 provincias</t>
         </is>
       </c>
       <c r="J313" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nacidos en España</t>
         </is>
       </c>
       <c r="K313" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>padrón, ECP, EPA (INE)</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>P2-E2: p de AKM0 frente a β = 0 ajustado (BH); el conjunto AKM0 puede no estar acotado aunque el p sea pequeño (primera etapa débil al nivel del shock)</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_15_34</t>
+          <t>F5_P3_EDUC_beta</t>
         </is>
       </c>
       <c r="B314" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C314" s="2" t="n"/>
-      <c r="D314" s="2" t="n"/>
+        <v>-0.169</v>
+      </c>
+      <c r="C314" s="2" t="n">
+        <v>-0.752</v>
+      </c>
+      <c r="D314" s="2" t="n">
+        <v>0.414</v>
+      </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>alumnos por profesor por punto porcentual</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -21915,46 +22061,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2016-2022</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>17 CCAA</t>
         </is>
       </c>
       <c r="J314" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>todos</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>EDUCAbase, ECP y padrón</t>
         </is>
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>P3 (educación): asociación entre el aumento de la población nacida fuera de 5-19 años y la ratio de alumnos por profesor en centros públicos (MC2E por comunidad; F efectivo = 39.5; p wild bootstrap de la forma reducida = 0.58; IC orientativo por errores agrupados en 17 comunidades)</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_35_54</t>
+          <t>F5_P5_HET_centro_y_este</t>
         </is>
       </c>
       <c r="B315" s="2" t="n">
-        <v>0.82</v>
+        <v>0.027</v>
       </c>
       <c r="C315" s="2" t="n"/>
       <c r="D315" s="2" t="n"/>
       <c r="E315" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -21962,46 +22113,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021-2024</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>NUTS2, centro y este</t>
         </is>
       </c>
       <c r="J315" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nativos</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Eurostat</t>
         </is>
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>P5, países centro y este: β leave-one-country-out (28 regiones; p wild bootstrap = 0.94)</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_HOSP_55_74</t>
+          <t>F5_P5_HET_continentales</t>
         </is>
       </c>
       <c r="B316" s="2" t="n">
-        <v>2.58</v>
+        <v>-0.163</v>
       </c>
       <c r="C316" s="2" t="n"/>
       <c r="D316" s="2" t="n"/>
       <c r="E316" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -22009,46 +22165,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021-2024</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>NUTS2, continentales</t>
         </is>
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nativos</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Eurostat</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>P5, países continentales: β leave-one-country-out (93 regiones; p wild bootstrap = 0.80)</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_15_34</t>
+          <t>F5_P5_HET_mediterráneos</t>
         </is>
       </c>
       <c r="B317" s="2" t="n">
-        <v>0.9</v>
+        <v>-0.501</v>
       </c>
       <c r="C317" s="2" t="n"/>
       <c r="D317" s="2" t="n"/>
       <c r="E317" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -22056,46 +22217,51 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021-2024</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>NUTS2, mediterráneos</t>
         </is>
       </c>
       <c r="J317" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nativos</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Eurostat</t>
         </is>
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+          <t>P5, países mediterráneos: β leave-one-country-out (57 regiones; p wild bootstrap = 0.31)</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_35_54</t>
+          <t>F5_P5_HET_nórdicos</t>
         </is>
       </c>
       <c r="B318" s="2" t="n">
-        <v>1.16</v>
+        <v>-0.904</v>
       </c>
       <c r="C318" s="2" t="n"/>
       <c r="D318" s="2" t="n"/>
       <c r="E318" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -22103,46 +22269,55 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021-2024</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>NUTS2, nórdicos</t>
         </is>
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nativos</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Eurostat</t>
         </is>
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+          <t>P5, países nórdicos: β leave-one-country-out (17 regiones; p wild bootstrap = 0.33)</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>F6_ENSE_RAZON_URG_55_74</t>
+          <t>F5_P5_beta</t>
         </is>
       </c>
       <c r="B319" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C319" s="2" t="n"/>
-      <c r="D319" s="2" t="n"/>
+        <v>-0.325</v>
+      </c>
+      <c r="C319" s="2" t="n">
+        <v>-0.968</v>
+      </c>
+      <c r="D319" s="2" t="n">
+        <v>0.318</v>
+      </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>razón (nativos = 1)</t>
+          <t>pp por pp</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -22150,56 +22325,61 @@
           <t>C4</t>
         </is>
       </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN</t>
+        </is>
+      </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021-2024</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>NUTS2 UE-27</t>
         </is>
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>nacidos fuera</t>
+          <t>nativos</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
         <is>
-          <t>ENSE 2017 (INE)</t>
+          <t>Eurostat (censo 2021, migr_imm3ctb, EU-LFS)</t>
         </is>
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+          <t>P5: asociación entre la llegada de población nacida fuera y la tasa de empleo de los nativos, NUTS2 de la UE-27, 2021-2024 (MC2E leave-one-country-out; p wild bootstrap por país = 0.38; IC orientativo por errores agrupados por país)</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>F6_POB_CUOTA_FUERA_ECV</t>
+          <t>F6_ENSE_RAZON_CONSULTAS_15_34</t>
         </is>
       </c>
       <c r="B320" s="2" t="n">
-        <v>18.5</v>
+        <v>1.02</v>
       </c>
       <c r="C320" s="2" t="n"/>
       <c r="D320" s="2" t="n"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>% de la población</t>
+          <t>razón (nativos = 1)</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -22214,39 +22394,39 @@
       </c>
       <c r="K320" t="inlineStr">
         <is>
-          <t>ECV (INE)</t>
+          <t>ENSE 2017 (INE)</t>
         </is>
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>Cuota de los nacidos fuera en la población de la ECV (hogares privados)</t>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_España</t>
+          <t>F6_ENSE_RAZON_CONSULTAS_35_54</t>
         </is>
       </c>
       <c r="B321" s="2" t="n">
-        <v>6252</v>
+        <v>0.84</v>
       </c>
       <c r="C321" s="2" t="n"/>
       <c r="D321" s="2" t="n"/>
       <c r="E321" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>razón (nativos = 1)</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -22256,44 +22436,44 @@
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>nacidos fuera</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>ENSE 2017 (INE)</t>
         </is>
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en España</t>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_Resto_UE</t>
+          <t>F6_ENSE_RAZON_CONSULTAS_55_74</t>
         </is>
       </c>
       <c r="B322" s="2" t="n">
-        <v>2813</v>
+        <v>0.96</v>
       </c>
       <c r="C322" s="2" t="n"/>
       <c r="D322" s="2" t="n"/>
       <c r="E322" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>razón (nativos = 1)</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -22303,44 +22483,44 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>Resto UE</t>
+          <t>nacidos fuera</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>ENSE 2017 (INE)</t>
         </is>
       </c>
       <c r="L322" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto UE</t>
+          <t>Uso relativo de consultas de primaria y especialista: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>F6_PREST_MONETARIAS_PC_Resto_del_mundo</t>
+          <t>F6_ENSE_RAZON_FAR_15_34</t>
         </is>
       </c>
       <c r="B323" s="2" t="n">
-        <v>1927</v>
+        <v>0.9</v>
       </c>
       <c r="C323" s="2" t="n"/>
       <c r="D323" s="2" t="n"/>
       <c r="E323" t="inlineStr">
         <is>
-          <t>€ por persona y año</t>
+          <t>razón (nativos = 1)</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -22350,44 +22530,44 @@
       </c>
       <c r="J323" t="inlineStr">
         <is>
-          <t>Resto del mundo</t>
+          <t>nacidos fuera</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>ENSE 2017 (INE)</t>
         </is>
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto del mundo</t>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>F6_PREST_NO_CONTRIB_CUOTA</t>
+          <t>F6_ENSE_RAZON_FAR_35_54</t>
         </is>
       </c>
       <c r="B324" s="2" t="n">
-        <v>2.5</v>
+        <v>0.89</v>
       </c>
       <c r="C324" s="2" t="n"/>
       <c r="D324" s="2" t="n"/>
       <c r="E324" t="inlineStr">
         <is>
-          <t>% de las prestaciones monetarias</t>
+          <t>razón (nativos = 1)</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="I324" t="inlineStr">
@@ -22397,62 +22577,626 @@
       </c>
       <c r="J324" t="inlineStr">
         <is>
-          <t>todos</t>
+          <t>nacidos fuera</t>
         </is>
       </c>
       <c r="K324" t="inlineStr">
         <is>
-          <t>ECV (INE) y Eurostat COFOG</t>
+          <t>ENSE 2017 (INE)</t>
         </is>
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>Rentas mínimas, IMV y ayudas a la vivienda sobre el total de prestaciones monetarias (calibradas a COFOG)</t>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>F6_TRABAJO_CUOTA_FUERA</t>
+          <t>F6_ENSE_RAZON_FAR_55_74</t>
         </is>
       </c>
       <c r="B325" s="2" t="n">
-        <v>15.5</v>
+        <v>0.85</v>
       </c>
       <c r="C325" s="2" t="n"/>
       <c r="D325" s="2" t="n"/>
       <c r="E325" t="inlineStr">
         <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Uso relativo de uso de medicamentos recetados: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_15_34</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C326" s="2" t="n"/>
+      <c r="D326" s="2" t="n"/>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_35_54</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="C327" s="2" t="n"/>
+      <c r="D327" s="2" t="n"/>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_HOSP_55_74</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="C328" s="2" t="n"/>
+      <c r="D328" s="2" t="n"/>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Uso relativo de días de hospital: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_15_34</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C329" s="2" t="n"/>
+      <c r="D329" s="2" t="n"/>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 15-34 años (n nacidos fuera = 655)</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_35_54</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="C330" s="2" t="n"/>
+      <c r="D330" s="2" t="n"/>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 35-54 años (n nacidos fuera = 1126)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>F6_ENSE_RAZON_URG_55_74</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C331" s="2" t="n"/>
+      <c r="D331" s="2" t="n"/>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>razón (nativos = 1)</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>ENSE 2017 (INE)</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Uso relativo de urgencias: nacidos fuera / nacidos en España, 55-74 años (n nacidos fuera = 389)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>F6_POB_CUOTA_FUERA_ECV</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C332" s="2" t="n"/>
+      <c r="D332" s="2" t="n"/>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>% de la población</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>nacidos fuera</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>ECV (INE)</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Cuota de los nacidos fuera en la población de la ECV (hogares privados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_España</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="n">
+        <v>6252</v>
+      </c>
+      <c r="C333" s="2" t="n"/>
+      <c r="D333" s="2" t="n"/>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en España</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_Resto_UE</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="n">
+        <v>2813</v>
+      </c>
+      <c r="C334" s="2" t="n"/>
+      <c r="D334" s="2" t="n"/>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Resto UE</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto UE</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>F6_PREST_MONETARIAS_PC_Resto_del_mundo</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="n">
+        <v>1927</v>
+      </c>
+      <c r="C335" s="2" t="n"/>
+      <c r="D335" s="2" t="n"/>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>€ por persona y año</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Resto del mundo</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Prestaciones monetarias por persona (calibradas a COFOG), nacidos en Resto del mundo</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>F6_PREST_NO_CONTRIB_CUOTA</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C336" s="2" t="n"/>
+      <c r="D336" s="2" t="n"/>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>% de las prestaciones monetarias</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>ECV (INE) y Eurostat COFOG</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Rentas mínimas, IMV y ayudas a la vivienda sobre el total de prestaciones monetarias (calibradas a COFOG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>F6_TRABAJO_CUOTA_FUERA</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C337" s="2" t="n"/>
+      <c r="D337" s="2" t="n"/>
+      <c r="E337" t="inlineStr">
+        <is>
           <t>% del total</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr">
+      <c r="F337" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="H325" t="inlineStr">
+      <c r="H337" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="I325" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="J325" t="inlineStr">
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
         <is>
           <t>nacidos fuera</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr">
+      <c r="K337" t="inlineStr">
         <is>
           <t>ECV (INE) y Eurostat</t>
         </is>
       </c>
-      <c r="L325" t="inlineStr">
+      <c r="L337" t="inlineStr">
         <is>
           <t>Cuota de los nacidos fuera en IRPF del trabajo y cotizaciones sociales (calibradas a las cuentas de las AAPP)</t>
         </is>

</xml_diff>

<commit_message>
Cierre: coherencia final (tablas, D11, lenguaje), estado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja66M5TMoQNzqNwDgvFAsk
</commit_message>
<xml_diff>
--- a/output/f7/tablas_m1.xlsx
+++ b/output/f7/tablas_m1.xlsx
@@ -9585,27 +9585,27 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Tasa de empleo</t>
+          <t>Tasa de empleo 16-64</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Tasa de paro</t>
+          <t>Tasa de paro (16 años o más)</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Temporalidad</t>
+          <t>Temporalidad (asalariados de 16 años o más)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Ocupados</t>
+          <t>Ocupados de 16 años o más (no dividir por la población 16-64)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Cuota de los ocupados</t>
+          <t>Cuota de los ocupados de 16 años o más</t>
         </is>
       </c>
     </row>

</xml_diff>